<commit_message>
WIP checkpoint 2026-08-24: inflation scripts, NFCe data, Excel updates
</commit_message>
<xml_diff>
--- a/data/financas2026-DataEntry.xlsx
+++ b/data/financas2026-DataEntry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardofgiovannini/Documents/GitHub/financas-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardofgiovannini/Documents/GitHub/financas-2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{368A67DE-6F83-184E-993B-D23260BBE6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE04CC7-A076-FA40-B77C-9F0EABF32CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33840" windowHeight="21600" firstSheet="2" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20340" yWindow="-20980" windowWidth="38400" windowHeight="20980" firstSheet="2" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 SYNC" sheetId="1" r:id="rId1"/>
@@ -2781,7 +2781,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3123,6 +3123,40 @@
     <xf numFmtId="0" fontId="42" fillId="19" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="48" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="48" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="48" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="48" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3171,43 +3205,6 @@
     <xf numFmtId="0" fontId="43" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="48" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="48" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="48" fillId="22" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="46" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5610,7 +5607,7 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="2700000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="2700000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -8214,10 +8211,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -8514,24 +8507,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
     </row>
     <row r="2" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
     </row>
     <row r="4" spans="2:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
@@ -8568,14 +8561,14 @@
       </c>
     </row>
     <row r="7" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="128" t="s">
+      <c r="B7" s="148" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="124"/>
-      <c r="D7" s="124"/>
-      <c r="E7" s="124"/>
-      <c r="F7" s="124"/>
-      <c r="G7" s="124"/>
+      <c r="C7" s="144"/>
+      <c r="D7" s="144"/>
+      <c r="E7" s="144"/>
+      <c r="F7" s="144"/>
+      <c r="G7" s="144"/>
     </row>
     <row r="8" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
@@ -8670,14 +8663,14 @@
       </c>
     </row>
     <row r="12" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="128" t="s">
+      <c r="B12" s="148" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="124"/>
-      <c r="D12" s="124"/>
-      <c r="E12" s="124"/>
-      <c r="F12" s="124"/>
-      <c r="G12" s="124"/>
+      <c r="C12" s="144"/>
+      <c r="D12" s="144"/>
+      <c r="E12" s="144"/>
+      <c r="F12" s="144"/>
+      <c r="G12" s="144"/>
     </row>
     <row r="13" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="5" t="s">
@@ -8726,14 +8719,14 @@
       </c>
     </row>
     <row r="15" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="128" t="s">
+      <c r="B15" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="124"/>
-      <c r="D15" s="124"/>
-      <c r="E15" s="124"/>
-      <c r="F15" s="124"/>
-      <c r="G15" s="124"/>
+      <c r="C15" s="144"/>
+      <c r="D15" s="144"/>
+      <c r="E15" s="144"/>
+      <c r="F15" s="144"/>
+      <c r="G15" s="144"/>
     </row>
     <row r="16" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="5" t="s">
@@ -8782,14 +8775,14 @@
       </c>
     </row>
     <row r="18" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="128" t="s">
+      <c r="B18" s="148" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="124"/>
-      <c r="D18" s="124"/>
-      <c r="E18" s="124"/>
-      <c r="F18" s="124"/>
-      <c r="G18" s="124"/>
+      <c r="C18" s="144"/>
+      <c r="D18" s="144"/>
+      <c r="E18" s="144"/>
+      <c r="F18" s="144"/>
+      <c r="G18" s="144"/>
     </row>
     <row r="19" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="5" t="s">
@@ -8838,14 +8831,14 @@
       </c>
     </row>
     <row r="21" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="128" t="s">
+      <c r="B21" s="148" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="124"/>
-      <c r="D21" s="124"/>
-      <c r="E21" s="124"/>
-      <c r="F21" s="124"/>
-      <c r="G21" s="124"/>
+      <c r="C21" s="144"/>
+      <c r="D21" s="144"/>
+      <c r="E21" s="144"/>
+      <c r="F21" s="144"/>
+      <c r="G21" s="144"/>
     </row>
     <row r="22" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="5" t="s">
@@ -8917,14 +8910,14 @@
       </c>
     </row>
     <row r="25" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="128" t="s">
+      <c r="B25" s="148" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="124"/>
-      <c r="D25" s="124"/>
-      <c r="E25" s="124"/>
-      <c r="F25" s="124"/>
-      <c r="G25" s="124"/>
+      <c r="C25" s="144"/>
+      <c r="D25" s="144"/>
+      <c r="E25" s="144"/>
+      <c r="F25" s="144"/>
+      <c r="G25" s="144"/>
     </row>
     <row r="26" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="5" t="s">
@@ -9019,24 +9012,24 @@
       </c>
     </row>
     <row r="31" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="125" t="s">
+      <c r="B31" s="145" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="124"/>
-      <c r="D31" s="124"/>
-      <c r="E31" s="124"/>
-      <c r="F31" s="124"/>
-      <c r="G31" s="124"/>
+      <c r="C31" s="144"/>
+      <c r="D31" s="144"/>
+      <c r="E31" s="144"/>
+      <c r="F31" s="144"/>
+      <c r="G31" s="144"/>
     </row>
     <row r="32" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="127" t="s">
+      <c r="B32" s="147" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="124"/>
-      <c r="D32" s="124"/>
-      <c r="E32" s="124"/>
-      <c r="F32" s="124"/>
-      <c r="G32" s="124"/>
+      <c r="C32" s="144"/>
+      <c r="D32" s="144"/>
+      <c r="E32" s="144"/>
+      <c r="F32" s="144"/>
+      <c r="G32" s="144"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
@@ -9112,36 +9105,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="158" t="s">
         <v>343</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
     </row>
     <row r="2" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="134" t="str">
+      <c r="A2" s="154" t="str">
         <f>"Total: R$"&amp;TEXT(SUM(D4:D149),"#,##0.00")</f>
         <v>Total: R$37,245.76</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="135" t="str">
+      <c r="B2" s="144"/>
+      <c r="C2" s="155" t="str">
         <f>COUNT(D4:D149)&amp;" transações"</f>
         <v>146 transações</v>
       </c>
-      <c r="D2" s="124"/>
-      <c r="E2" s="137" t="s">
+      <c r="D2" s="144"/>
+      <c r="E2" s="157" t="s">
         <v>344</v>
       </c>
-      <c r="F2" s="124"/>
-      <c r="G2" s="136" t="s">
+      <c r="F2" s="144"/>
+      <c r="G2" s="156" t="s">
         <v>345</v>
       </c>
-      <c r="H2" s="124"/>
+      <c r="H2" s="144"/>
     </row>
     <row r="3" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="112" t="s">
@@ -13012,33 +13005,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="139" t="s">
+      <c r="A1" s="159" t="s">
         <v>547</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
     </row>
     <row r="2" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="137" t="str">
+      <c r="A2" s="157" t="str">
         <f>"ML Entregues: R$"&amp;TEXT(SUMIFS(D4:D72,B4:B72,"Mercado Livre",F4:F72,"delivered"),"#,##0.00")</f>
         <v>ML Entregues: R$25,793.43</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="140" t="str">
+      <c r="B2" s="144"/>
+      <c r="C2" s="160" t="str">
         <f>"iFood: R$"&amp;TEXT(SUMIFS(D4:D72,B4:B72,"iFood"),"#,##0.00")&amp;" ("&amp;COUNTIF(B4:B72,"iFood")&amp;" pedidos, "&amp;COUNTIFS(B4:B72,"iFood",D4:D72,"&gt;0")&amp;" com valor)"</f>
         <v>iFood: R$847.65 (13 pedidos, 9 com valor)</v>
       </c>
-      <c r="D2" s="124"/>
-      <c r="E2" s="134" t="str">
+      <c r="D2" s="144"/>
+      <c r="E2" s="154" t="str">
         <f>"Total Combinado: R$"&amp;TEXT(SUMIFS(D4:D72,B4:B72,"Mercado Livre",F4:F72,"delivered")+SUMIFS(D4:D72,B4:B72,"iFood"),"#,##0.00")</f>
         <v>Total Combinado: R$26,641.08</v>
       </c>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
     </row>
     <row r="3" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="112" t="s">
@@ -14709,1273 +14702,1266 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="141" t="s">
+      <c r="A1" s="139" t="s">
         <v>661</v>
       </c>
-      <c r="B1" s="142"/>
-      <c r="C1" s="142"/>
-      <c r="D1" s="142"/>
-      <c r="E1" s="142"/>
-      <c r="F1" s="142"/>
-      <c r="G1" s="142"/>
-      <c r="H1" s="142"/>
-      <c r="I1" s="142"/>
-      <c r="J1" s="142"/>
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="143" t="s">
+      <c r="A2" s="140" t="s">
         <v>676</v>
       </c>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="141"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="141"/>
+      <c r="H2" s="141"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="141"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="144"/>
-      <c r="B3" s="144"/>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
-      <c r="H3" s="144"/>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
+      <c r="A3" s="123"/>
+      <c r="B3" s="123"/>
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="145" t="s">
+      <c r="A4" s="134" t="s">
         <v>662</v>
       </c>
-      <c r="B4" s="142"/>
-      <c r="C4" s="142"/>
-      <c r="D4" s="142"/>
-      <c r="E4" s="142"/>
-      <c r="F4" s="142"/>
-      <c r="G4" s="142"/>
-      <c r="H4" s="142"/>
-      <c r="I4" s="142"/>
-      <c r="J4" s="142"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="136"/>
+      <c r="F4" s="136"/>
+      <c r="G4" s="136"/>
+      <c r="H4" s="136"/>
+      <c r="I4" s="136"/>
+      <c r="J4" s="136"/>
     </row>
     <row r="5" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="141" t="s">
         <v>678</v>
       </c>
-      <c r="B5" s="146"/>
-      <c r="C5" s="146"/>
-      <c r="D5" s="146"/>
-      <c r="E5" s="146"/>
-      <c r="F5" s="146"/>
-      <c r="G5" s="146"/>
-      <c r="H5" s="146"/>
-      <c r="I5" s="146"/>
-      <c r="J5" s="146"/>
+      <c r="B5" s="141"/>
+      <c r="C5" s="141"/>
+      <c r="D5" s="141"/>
+      <c r="E5" s="141"/>
+      <c r="F5" s="141"/>
+      <c r="G5" s="141"/>
+      <c r="H5" s="141"/>
+      <c r="I5" s="141"/>
+      <c r="J5" s="141"/>
     </row>
     <row r="6" spans="1:10" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="146"/>
-      <c r="B6" s="146"/>
-      <c r="C6" s="146"/>
-      <c r="D6" s="146"/>
-      <c r="E6" s="146"/>
-      <c r="F6" s="146"/>
-      <c r="G6" s="146"/>
-      <c r="H6" s="146"/>
-      <c r="I6" s="146"/>
-      <c r="J6" s="146"/>
+      <c r="A6" s="141"/>
+      <c r="B6" s="141"/>
+      <c r="C6" s="141"/>
+      <c r="D6" s="141"/>
+      <c r="E6" s="141"/>
+      <c r="F6" s="141"/>
+      <c r="G6" s="141"/>
+      <c r="H6" s="141"/>
+      <c r="I6" s="141"/>
+      <c r="J6" s="141"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="144"/>
-      <c r="B7" s="144"/>
-      <c r="C7" s="144"/>
-      <c r="D7" s="144"/>
-      <c r="E7" s="144"/>
-      <c r="F7" s="144"/>
-      <c r="G7" s="144"/>
-      <c r="H7" s="144"/>
-      <c r="I7" s="144"/>
-      <c r="J7" s="144"/>
+      <c r="A7" s="123"/>
+      <c r="B7" s="123"/>
+      <c r="C7" s="123"/>
+      <c r="D7" s="123"/>
+      <c r="E7" s="123"/>
+      <c r="F7" s="123"/>
+      <c r="G7" s="123"/>
+      <c r="H7" s="123"/>
+      <c r="I7" s="123"/>
+      <c r="J7" s="123"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="147" t="s">
+      <c r="A8" s="142" t="s">
         <v>663</v>
       </c>
-      <c r="B8" s="147"/>
-      <c r="C8" s="147" t="s">
+      <c r="B8" s="142"/>
+      <c r="C8" s="142" t="s">
         <v>664</v>
       </c>
-      <c r="D8" s="147"/>
-      <c r="E8" s="147" t="s">
+      <c r="D8" s="142"/>
+      <c r="E8" s="142" t="s">
         <v>665</v>
       </c>
-      <c r="F8" s="147"/>
-      <c r="G8" s="148" t="s">
+      <c r="F8" s="142"/>
+      <c r="G8" s="142" t="s">
         <v>666</v>
       </c>
-      <c r="H8" s="148"/>
-      <c r="I8" s="148" t="s">
+      <c r="H8" s="142"/>
+      <c r="I8" s="142" t="s">
         <v>667</v>
       </c>
-      <c r="J8" s="148"/>
+      <c r="J8" s="142"/>
     </row>
     <row r="9" spans="1:10" ht="22" x14ac:dyDescent="0.3">
-      <c r="A9" s="149">
+      <c r="A9" s="138">
         <f>SUM('💳 MP Faturas'!D4:D149)</f>
         <v>37245.759999999987</v>
       </c>
-      <c r="B9" s="149"/>
-      <c r="C9" s="149">
+      <c r="B9" s="138"/>
+      <c r="C9" s="138">
         <f>'🏦 Banks'!C9</f>
         <v>23196.899999999998</v>
       </c>
-      <c r="D9" s="149"/>
-      <c r="E9" s="149">
+      <c r="D9" s="138"/>
+      <c r="E9" s="138">
         <f>'🔄 Subscriptions'!I21</f>
         <v>365.79999999999995</v>
       </c>
-      <c r="F9" s="149"/>
-      <c r="G9" s="149">
+      <c r="F9" s="138"/>
+      <c r="G9" s="138">
         <f>E9*12</f>
         <v>4389.5999999999995</v>
       </c>
-      <c r="H9" s="149"/>
-      <c r="I9" s="149">
+      <c r="H9" s="138"/>
+      <c r="I9" s="138">
         <f>SUM('🌍 International'!F4:F35)</f>
         <v>1144313.82</v>
       </c>
-      <c r="J9" s="149"/>
+      <c r="J9" s="138"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="144"/>
-      <c r="B10" s="144"/>
-      <c r="C10" s="144"/>
-      <c r="D10" s="144"/>
-      <c r="E10" s="144"/>
-      <c r="F10" s="144"/>
-      <c r="G10" s="144"/>
-      <c r="H10" s="144"/>
-      <c r="I10" s="144"/>
-      <c r="J10" s="144"/>
+      <c r="A10" s="123"/>
+      <c r="B10" s="123"/>
+      <c r="C10" s="123"/>
+      <c r="D10" s="123"/>
+      <c r="E10" s="123"/>
+      <c r="F10" s="123"/>
+      <c r="G10" s="123"/>
+      <c r="H10" s="123"/>
+      <c r="I10" s="123"/>
+      <c r="J10" s="123"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="144"/>
-      <c r="B11" s="144"/>
-      <c r="C11" s="144"/>
-      <c r="D11" s="144"/>
-      <c r="E11" s="144"/>
-      <c r="F11" s="144"/>
-      <c r="G11" s="144"/>
-      <c r="H11" s="144"/>
-      <c r="I11" s="144"/>
-      <c r="J11" s="144"/>
+      <c r="A11" s="123"/>
+      <c r="B11" s="123"/>
+      <c r="C11" s="123"/>
+      <c r="D11" s="123"/>
+      <c r="E11" s="123"/>
+      <c r="F11" s="123"/>
+      <c r="G11" s="123"/>
+      <c r="H11" s="123"/>
+      <c r="I11" s="123"/>
+      <c r="J11" s="123"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="145" t="s">
+      <c r="A12" s="134" t="s">
         <v>668</v>
       </c>
-      <c r="B12" s="142"/>
-      <c r="C12" s="142"/>
-      <c r="D12" s="144"/>
-      <c r="E12" s="145" t="s">
+      <c r="B12" s="136"/>
+      <c r="C12" s="136"/>
+      <c r="D12" s="123"/>
+      <c r="E12" s="134" t="s">
         <v>670</v>
       </c>
-      <c r="F12" s="142"/>
-      <c r="G12" s="142"/>
-      <c r="H12" s="144"/>
-      <c r="I12" s="144"/>
-      <c r="J12" s="144"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="136"/>
+      <c r="H12" s="123"/>
+      <c r="I12" s="123"/>
+      <c r="J12" s="123"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="150" t="s">
+      <c r="A13" s="124" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="150" t="s">
+      <c r="B13" s="124" t="s">
         <v>669</v>
       </c>
-      <c r="C13" s="150" t="s">
+      <c r="C13" s="124" t="s">
         <v>677</v>
       </c>
-      <c r="D13" s="144"/>
-      <c r="E13" s="150" t="s">
+      <c r="D13" s="123"/>
+      <c r="E13" s="124" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="150" t="s">
+      <c r="F13" s="124" t="s">
         <v>176</v>
       </c>
-      <c r="G13" s="150" t="s">
+      <c r="G13" s="124" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="144"/>
-      <c r="I13" s="144"/>
-      <c r="J13" s="144"/>
+      <c r="H13" s="123"/>
+      <c r="I13" s="123"/>
+      <c r="J13" s="123"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="151" t="s">
+      <c r="A14" s="125" t="s">
         <v>435</v>
       </c>
-      <c r="B14" s="152">
+      <c r="B14" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A14,'💳 MP Faturas'!D4:D149)</f>
         <v>9036.83</v>
       </c>
-      <c r="C14" s="153">
-        <f>B14/SUM($B$14:$B$20)</f>
+      <c r="C14" s="127">
+        <f t="shared" ref="C14:C20" si="0">B14/SUM($B$14:$B$20)</f>
         <v>0.25286921152402381</v>
       </c>
-      <c r="D14" s="144"/>
-      <c r="E14" s="151" t="s">
+      <c r="D14" s="123"/>
+      <c r="E14" s="125" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="152">
+      <c r="F14" s="126">
         <f>SUMIF('🔄 Subscriptions'!L:L,E14,'🔄 Subscriptions'!I:I)</f>
         <v>331.8</v>
       </c>
-      <c r="G14" s="154">
+      <c r="G14" s="128">
         <f>COUNTIF('🔄 Subscriptions'!L:L,E14)</f>
         <v>4</v>
       </c>
-      <c r="H14" s="144"/>
-      <c r="I14" s="144"/>
-      <c r="J14" s="144"/>
+      <c r="H14" s="123"/>
+      <c r="I14" s="123"/>
+      <c r="J14" s="123"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="151" t="s">
+      <c r="A15" s="125" t="s">
         <v>401</v>
       </c>
-      <c r="B15" s="152">
+      <c r="B15" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A15,'💳 MP Faturas'!D4:D149)</f>
         <v>8744.6799999999985</v>
       </c>
-      <c r="C15" s="153">
-        <f>B15/SUM($B$14:$B$20)</f>
+      <c r="C15" s="127">
+        <f t="shared" si="0"/>
         <v>0.2446942497125541</v>
       </c>
-      <c r="D15" s="144"/>
-      <c r="E15" s="151" t="s">
+      <c r="D15" s="123"/>
+      <c r="E15" s="125" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="152">
+      <c r="F15" s="126">
         <f>SUMIF('🔄 Subscriptions'!L:L,E15,'🔄 Subscriptions'!I:I)</f>
         <v>365.79999999999995</v>
       </c>
-      <c r="G15" s="154">
+      <c r="G15" s="128">
         <f>COUNTIF('🔄 Subscriptions'!L:L,E15)</f>
         <v>4</v>
       </c>
-      <c r="H15" s="144"/>
-      <c r="I15" s="144"/>
-      <c r="J15" s="144"/>
+      <c r="H15" s="123"/>
+      <c r="I15" s="123"/>
+      <c r="J15" s="123"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="151" t="s">
+      <c r="A16" s="125" t="s">
         <v>360</v>
       </c>
-      <c r="B16" s="152">
+      <c r="B16" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A16,'💳 MP Faturas'!D4:D149)</f>
         <v>6624.3600000000015</v>
       </c>
-      <c r="C16" s="153">
-        <f>B16/SUM($B$14:$B$20)</f>
+      <c r="C16" s="127">
+        <f t="shared" si="0"/>
         <v>0.1853633066076581</v>
       </c>
-      <c r="D16" s="144"/>
-      <c r="E16" s="151" t="s">
+      <c r="D16" s="123"/>
+      <c r="E16" s="125" t="s">
         <v>83</v>
       </c>
-      <c r="F16" s="152">
+      <c r="F16" s="126">
         <f>SUMIF('🔄 Subscriptions'!L:L,E16,'🔄 Subscriptions'!I:I)</f>
         <v>646.93999999999994</v>
       </c>
-      <c r="G16" s="154">
+      <c r="G16" s="128">
         <f>COUNTIF('🔄 Subscriptions'!L:L,E16)</f>
         <v>7</v>
       </c>
-      <c r="H16" s="144"/>
-      <c r="I16" s="144"/>
-      <c r="J16" s="144"/>
+      <c r="H16" s="123"/>
+      <c r="I16" s="123"/>
+      <c r="J16" s="123"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="151" t="s">
+      <c r="A17" s="125" t="s">
         <v>376</v>
       </c>
-      <c r="B17" s="152">
+      <c r="B17" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A17,'💳 MP Faturas'!D4:D149)</f>
         <v>6455.1</v>
       </c>
-      <c r="C17" s="153">
-        <f>B17/SUM($B$14:$B$20)</f>
+      <c r="C17" s="127">
+        <f t="shared" si="0"/>
         <v>0.18062706140413468</v>
       </c>
-      <c r="D17" s="144"/>
-      <c r="E17" s="144"/>
-      <c r="F17" s="155"/>
-      <c r="G17" s="156"/>
-      <c r="H17" s="144"/>
-      <c r="I17" s="144"/>
-      <c r="J17" s="144"/>
+      <c r="D17" s="123"/>
+      <c r="E17" s="123"/>
+      <c r="F17" s="129"/>
+      <c r="G17" s="130"/>
+      <c r="H17" s="123"/>
+      <c r="I17" s="123"/>
+      <c r="J17" s="123"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="151" t="s">
+      <c r="A18" s="125" t="s">
         <v>368</v>
       </c>
-      <c r="B18" s="152">
+      <c r="B18" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A18,'💳 MP Faturas'!D4:D149)</f>
         <v>2235.58</v>
       </c>
-      <c r="C18" s="153">
-        <f>B18/SUM($B$14:$B$20)</f>
+      <c r="C18" s="127">
+        <f t="shared" si="0"/>
         <v>6.2556156517150061E-2</v>
       </c>
-      <c r="D18" s="144"/>
-      <c r="E18" s="144"/>
-      <c r="F18" s="155"/>
-      <c r="G18" s="156"/>
-      <c r="H18" s="144"/>
-      <c r="I18" s="144"/>
-      <c r="J18" s="144"/>
+      <c r="D18" s="123"/>
+      <c r="E18" s="123"/>
+      <c r="F18" s="129"/>
+      <c r="G18" s="130"/>
+      <c r="H18" s="123"/>
+      <c r="I18" s="123"/>
+      <c r="J18" s="123"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" s="151" t="s">
+      <c r="A19" s="125" t="s">
         <v>373</v>
       </c>
-      <c r="B19" s="152">
+      <c r="B19" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A19,'💳 MP Faturas'!D4:D149)</f>
         <v>1413.1200000000001</v>
       </c>
-      <c r="C19" s="153">
-        <f>B19/SUM($B$14:$B$20)</f>
+      <c r="C19" s="127">
+        <f t="shared" si="0"/>
         <v>3.954202305330836E-2</v>
       </c>
-      <c r="D19" s="144"/>
-      <c r="E19" s="144"/>
-      <c r="F19" s="155"/>
-      <c r="G19" s="156"/>
-      <c r="H19" s="144"/>
-      <c r="I19" s="144"/>
-      <c r="J19" s="144"/>
+      <c r="D19" s="123"/>
+      <c r="E19" s="123"/>
+      <c r="F19" s="129"/>
+      <c r="G19" s="130"/>
+      <c r="H19" s="123"/>
+      <c r="I19" s="123"/>
+      <c r="J19" s="123"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="151" t="s">
+      <c r="A20" s="125" t="s">
         <v>363</v>
       </c>
-      <c r="B20" s="152">
+      <c r="B20" s="126">
         <f>SUMIF('💳 MP Faturas'!E4:E149,A20,'💳 MP Faturas'!D4:D149)</f>
         <v>1227.5</v>
       </c>
-      <c r="C20" s="153">
-        <f>B20/SUM($B$14:$B$20)</f>
+      <c r="C20" s="127">
+        <f t="shared" si="0"/>
         <v>3.4347991181170746E-2</v>
       </c>
-      <c r="D20" s="144"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="155"/>
-      <c r="G20" s="156"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="144"/>
-      <c r="J20" s="144"/>
+      <c r="D20" s="123"/>
+      <c r="E20" s="123"/>
+      <c r="F20" s="129"/>
+      <c r="G20" s="130"/>
+      <c r="H20" s="123"/>
+      <c r="I20" s="123"/>
+      <c r="J20" s="123"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="144"/>
-      <c r="B21" s="155"/>
-      <c r="C21" s="144"/>
-      <c r="D21" s="144"/>
-      <c r="E21" s="144"/>
-      <c r="F21" s="155"/>
-      <c r="G21" s="156"/>
-      <c r="H21" s="144"/>
-      <c r="I21" s="144"/>
-      <c r="J21" s="144"/>
+      <c r="A21" s="123"/>
+      <c r="B21" s="129"/>
+      <c r="C21" s="123"/>
+      <c r="D21" s="123"/>
+      <c r="E21" s="123"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="130"/>
+      <c r="H21" s="123"/>
+      <c r="I21" s="123"/>
+      <c r="J21" s="123"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="144"/>
-      <c r="B22" s="155"/>
-      <c r="C22" s="144"/>
-      <c r="D22" s="144"/>
-      <c r="E22" s="144"/>
-      <c r="F22" s="155"/>
-      <c r="G22" s="156"/>
-      <c r="H22" s="144"/>
-      <c r="I22" s="144"/>
-      <c r="J22" s="144"/>
+      <c r="A22" s="123"/>
+      <c r="B22" s="129"/>
+      <c r="C22" s="123"/>
+      <c r="D22" s="123"/>
+      <c r="E22" s="123"/>
+      <c r="F22" s="129"/>
+      <c r="G22" s="130"/>
+      <c r="H22" s="123"/>
+      <c r="I22" s="123"/>
+      <c r="J22" s="123"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="144"/>
-      <c r="B23" s="155"/>
-      <c r="C23" s="144"/>
-      <c r="D23" s="144"/>
-      <c r="E23" s="144"/>
-      <c r="F23" s="155"/>
-      <c r="G23" s="156"/>
-      <c r="H23" s="144"/>
-      <c r="I23" s="144"/>
-      <c r="J23" s="144"/>
+      <c r="A23" s="123"/>
+      <c r="B23" s="129"/>
+      <c r="C23" s="123"/>
+      <c r="D23" s="123"/>
+      <c r="E23" s="123"/>
+      <c r="F23" s="129"/>
+      <c r="G23" s="130"/>
+      <c r="H23" s="123"/>
+      <c r="I23" s="123"/>
+      <c r="J23" s="123"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="145" t="s">
+      <c r="A24" s="134" t="s">
         <v>671</v>
       </c>
-      <c r="B24" s="157"/>
-      <c r="C24" s="142"/>
-      <c r="D24" s="144"/>
-      <c r="E24" s="145" t="s">
+      <c r="B24" s="135"/>
+      <c r="C24" s="136"/>
+      <c r="D24" s="123"/>
+      <c r="E24" s="134" t="s">
         <v>672</v>
       </c>
-      <c r="F24" s="157"/>
-      <c r="G24" s="158"/>
-      <c r="H24" s="144"/>
-      <c r="I24" s="144"/>
-      <c r="J24" s="144"/>
+      <c r="F24" s="135"/>
+      <c r="G24" s="137"/>
+      <c r="H24" s="123"/>
+      <c r="I24" s="123"/>
+      <c r="J24" s="123"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="150" t="s">
+      <c r="A25" s="124" t="s">
         <v>329</v>
       </c>
-      <c r="B25" s="159" t="s">
+      <c r="B25" s="131" t="s">
         <v>669</v>
       </c>
-      <c r="C25" s="150" t="s">
+      <c r="C25" s="124" t="s">
         <v>332</v>
       </c>
-      <c r="D25" s="144"/>
-      <c r="E25" s="150" t="s">
+      <c r="D25" s="123"/>
+      <c r="E25" s="124" t="s">
         <v>291</v>
       </c>
-      <c r="F25" s="159" t="s">
+      <c r="F25" s="131" t="s">
         <v>290</v>
       </c>
-      <c r="G25" s="160" t="s">
+      <c r="G25" s="132" t="s">
         <v>673</v>
       </c>
-      <c r="H25" s="144"/>
-      <c r="I25" s="144"/>
-      <c r="J25" s="144"/>
+      <c r="H25" s="123"/>
+      <c r="I25" s="123"/>
+      <c r="J25" s="123"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="161">
+      <c r="A26" s="133">
         <f>'📅 Weekly'!C4</f>
         <v>46027</v>
       </c>
-      <c r="B26" s="152">
+      <c r="B26" s="126">
         <f>ABS('📅 Weekly'!E4)</f>
         <v>1032.06</v>
       </c>
-      <c r="C26" s="154">
+      <c r="C26" s="128">
         <f>'📅 Weekly'!F4</f>
         <v>14</v>
       </c>
-      <c r="D26" s="144"/>
-      <c r="E26" s="151" t="s">
+      <c r="D26" s="123"/>
+      <c r="E26" s="125" t="s">
         <v>299</v>
       </c>
-      <c r="F26" s="152">
+      <c r="F26" s="126">
         <f>SUMIF('🌍 International'!H4:H35,E26,'🌍 International'!F4:F35)</f>
         <v>652788.61</v>
       </c>
-      <c r="G26" s="154">
+      <c r="G26" s="128">
         <f>COUNTIF('🌍 International'!H4:H35,E26)</f>
         <v>19</v>
       </c>
-      <c r="H26" s="144"/>
-      <c r="I26" s="144"/>
-      <c r="J26" s="144"/>
+      <c r="H26" s="123"/>
+      <c r="I26" s="123"/>
+      <c r="J26" s="123"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="161">
+      <c r="A27" s="133">
         <f>'📅 Weekly'!C5</f>
         <v>46034</v>
       </c>
-      <c r="B27" s="152">
+      <c r="B27" s="126">
         <f>ABS('📅 Weekly'!E5)</f>
         <v>137.16</v>
       </c>
-      <c r="C27" s="154">
+      <c r="C27" s="128">
         <f>'📅 Weekly'!F5</f>
         <v>2</v>
       </c>
-      <c r="D27" s="144"/>
-      <c r="E27" s="151" t="s">
+      <c r="D27" s="123"/>
+      <c r="E27" s="125" t="s">
         <v>296</v>
       </c>
-      <c r="F27" s="152">
+      <c r="F27" s="126">
         <f>SUMIF('🌍 International'!H4:H35,E27,'🌍 International'!F4:F35)</f>
         <v>197706.57</v>
       </c>
-      <c r="G27" s="154">
+      <c r="G27" s="128">
         <f>COUNTIF('🌍 International'!H4:H35,E27)</f>
         <v>7</v>
       </c>
-      <c r="H27" s="144"/>
-      <c r="I27" s="144"/>
-      <c r="J27" s="144"/>
+      <c r="H27" s="123"/>
+      <c r="I27" s="123"/>
+      <c r="J27" s="123"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="161">
+      <c r="A28" s="133">
         <f>'📅 Weekly'!C6</f>
         <v>46041</v>
       </c>
-      <c r="B28" s="152">
+      <c r="B28" s="126">
         <f>ABS('📅 Weekly'!E6)</f>
         <v>1806.44</v>
       </c>
-      <c r="C28" s="154">
+      <c r="C28" s="128">
         <f>'📅 Weekly'!F6</f>
         <v>3</v>
       </c>
-      <c r="D28" s="144"/>
-      <c r="E28" s="151" t="s">
+      <c r="D28" s="123"/>
+      <c r="E28" s="125" t="s">
         <v>307</v>
       </c>
-      <c r="F28" s="152">
+      <c r="F28" s="126">
         <f>SUMIF('🌍 International'!H4:H35,E28,'🌍 International'!F4:F35)</f>
         <v>175765.83000000002</v>
       </c>
-      <c r="G28" s="154">
+      <c r="G28" s="128">
         <f>COUNTIF('🌍 International'!H4:H35,E28)</f>
         <v>3</v>
       </c>
-      <c r="H28" s="144"/>
-      <c r="I28" s="144"/>
-      <c r="J28" s="144"/>
+      <c r="H28" s="123"/>
+      <c r="I28" s="123"/>
+      <c r="J28" s="123"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="161">
+      <c r="A29" s="133">
         <f>'📅 Weekly'!C7</f>
         <v>46048</v>
       </c>
-      <c r="B29" s="152">
+      <c r="B29" s="126">
         <f>ABS('📅 Weekly'!E7)</f>
         <v>624.53</v>
       </c>
-      <c r="C29" s="154">
+      <c r="C29" s="128">
         <f>'📅 Weekly'!F7</f>
         <v>2</v>
       </c>
-      <c r="D29" s="144"/>
-      <c r="E29" s="151" t="s">
+      <c r="D29" s="123"/>
+      <c r="E29" s="125" t="s">
         <v>310</v>
       </c>
-      <c r="F29" s="152">
+      <c r="F29" s="126">
         <f>SUMIF('🌍 International'!H4:H35,E29,'🌍 International'!F4:F35)</f>
         <v>98857</v>
       </c>
-      <c r="G29" s="154">
+      <c r="G29" s="128">
         <f>COUNTIF('🌍 International'!H4:H35,E29)</f>
         <v>2</v>
       </c>
-      <c r="H29" s="144"/>
-      <c r="I29" s="144"/>
-      <c r="J29" s="144"/>
+      <c r="H29" s="123"/>
+      <c r="I29" s="123"/>
+      <c r="J29" s="123"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="161">
+      <c r="A30" s="133">
         <f>'📅 Weekly'!C8</f>
         <v>46055</v>
       </c>
-      <c r="B30" s="152">
+      <c r="B30" s="126">
         <f>ABS('📅 Weekly'!E8)</f>
         <v>402.99999999999989</v>
       </c>
-      <c r="C30" s="154">
+      <c r="C30" s="128">
         <f>'📅 Weekly'!F8</f>
         <v>3</v>
       </c>
-      <c r="D30" s="144"/>
-      <c r="E30" s="151" t="s">
+      <c r="D30" s="123"/>
+      <c r="E30" s="125" t="s">
         <v>315</v>
       </c>
-      <c r="F30" s="152">
+      <c r="F30" s="126">
         <f>SUMIF('🌍 International'!H4:H35,E30,'🌍 International'!F4:F35)</f>
         <v>19195.810000000001</v>
       </c>
-      <c r="G30" s="154">
+      <c r="G30" s="128">
         <f>COUNTIF('🌍 International'!H4:H35,E30)</f>
         <v>1</v>
       </c>
-      <c r="H30" s="144"/>
-      <c r="I30" s="144"/>
-      <c r="J30" s="144"/>
+      <c r="H30" s="123"/>
+      <c r="I30" s="123"/>
+      <c r="J30" s="123"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" s="161">
+      <c r="A31" s="133">
         <f>'📅 Weekly'!C9</f>
         <v>46062</v>
       </c>
-      <c r="B31" s="152">
+      <c r="B31" s="126">
         <f>ABS('📅 Weekly'!E9)</f>
         <v>71.650000000000006</v>
       </c>
-      <c r="C31" s="154">
+      <c r="C31" s="128">
         <f>'📅 Weekly'!F9</f>
         <v>2</v>
       </c>
-      <c r="D31" s="144"/>
-      <c r="E31" s="151"/>
-      <c r="F31" s="152"/>
-      <c r="G31" s="154"/>
-      <c r="H31" s="144"/>
-      <c r="I31" s="144"/>
-      <c r="J31" s="144"/>
+      <c r="D31" s="123"/>
+      <c r="E31" s="125"/>
+      <c r="F31" s="126"/>
+      <c r="G31" s="128"/>
+      <c r="H31" s="123"/>
+      <c r="I31" s="123"/>
+      <c r="J31" s="123"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" s="161">
+      <c r="A32" s="133">
         <f>'📅 Weekly'!C10</f>
         <v>46069</v>
       </c>
-      <c r="B32" s="152">
+      <c r="B32" s="126">
         <f>ABS('📅 Weekly'!E10)</f>
         <v>646.47</v>
       </c>
-      <c r="C32" s="154">
+      <c r="C32" s="128">
         <f>'📅 Weekly'!F10</f>
         <v>2</v>
       </c>
-      <c r="D32" s="144"/>
-      <c r="E32" s="144"/>
-      <c r="F32" s="155"/>
-      <c r="G32" s="156"/>
-      <c r="H32" s="144"/>
-      <c r="I32" s="144"/>
-      <c r="J32" s="144"/>
+      <c r="D32" s="123"/>
+      <c r="E32" s="123"/>
+      <c r="F32" s="129"/>
+      <c r="G32" s="130"/>
+      <c r="H32" s="123"/>
+      <c r="I32" s="123"/>
+      <c r="J32" s="123"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" s="161">
+      <c r="A33" s="133">
         <f>'📅 Weekly'!C11</f>
         <v>46076</v>
       </c>
-      <c r="B33" s="152">
+      <c r="B33" s="126">
         <f>ABS('📅 Weekly'!E11)</f>
         <v>99.9</v>
       </c>
-      <c r="C33" s="154">
+      <c r="C33" s="128">
         <f>'📅 Weekly'!F11</f>
         <v>1</v>
       </c>
-      <c r="D33" s="144"/>
-      <c r="E33" s="144"/>
-      <c r="F33" s="155"/>
-      <c r="G33" s="156"/>
-      <c r="H33" s="144"/>
-      <c r="I33" s="144"/>
-      <c r="J33" s="144"/>
+      <c r="D33" s="123"/>
+      <c r="E33" s="123"/>
+      <c r="F33" s="129"/>
+      <c r="G33" s="130"/>
+      <c r="H33" s="123"/>
+      <c r="I33" s="123"/>
+      <c r="J33" s="123"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" s="161">
+      <c r="A34" s="133">
         <f>'📅 Weekly'!C12</f>
         <v>46083</v>
       </c>
-      <c r="B34" s="152">
+      <c r="B34" s="126">
         <f>ABS('📅 Weekly'!E12)</f>
         <v>185.13</v>
       </c>
-      <c r="C34" s="154">
+      <c r="C34" s="128">
         <f>'📅 Weekly'!F12</f>
         <v>3</v>
       </c>
-      <c r="D34" s="144"/>
-      <c r="E34" s="144"/>
-      <c r="F34" s="155"/>
-      <c r="G34" s="156"/>
-      <c r="H34" s="144"/>
-      <c r="I34" s="144"/>
-      <c r="J34" s="144"/>
+      <c r="D34" s="123"/>
+      <c r="E34" s="123"/>
+      <c r="F34" s="129"/>
+      <c r="G34" s="130"/>
+      <c r="H34" s="123"/>
+      <c r="I34" s="123"/>
+      <c r="J34" s="123"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="161">
+      <c r="A35" s="133">
         <f>'📅 Weekly'!C13</f>
         <v>46090</v>
       </c>
-      <c r="B35" s="152">
+      <c r="B35" s="126">
         <f>ABS('📅 Weekly'!E13)</f>
         <v>133.68</v>
       </c>
-      <c r="C35" s="154">
+      <c r="C35" s="128">
         <f>'📅 Weekly'!F13</f>
         <v>2</v>
       </c>
-      <c r="D35" s="144"/>
-      <c r="E35" s="144"/>
-      <c r="F35" s="155"/>
-      <c r="G35" s="156"/>
-      <c r="H35" s="144"/>
-      <c r="I35" s="144"/>
-      <c r="J35" s="144"/>
+      <c r="D35" s="123"/>
+      <c r="E35" s="123"/>
+      <c r="F35" s="129"/>
+      <c r="G35" s="130"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="123"/>
+      <c r="J35" s="123"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A36" s="161">
+      <c r="A36" s="133">
         <f>'📅 Weekly'!C14</f>
         <v>46097</v>
       </c>
-      <c r="B36" s="152">
+      <c r="B36" s="126">
         <f>ABS('📅 Weekly'!E14)</f>
         <v>752.36</v>
       </c>
-      <c r="C36" s="154">
+      <c r="C36" s="128">
         <f>'📅 Weekly'!F14</f>
         <v>3</v>
       </c>
-      <c r="D36" s="144"/>
-      <c r="E36" s="144"/>
-      <c r="F36" s="155"/>
-      <c r="G36" s="156"/>
-      <c r="H36" s="144"/>
-      <c r="I36" s="144"/>
-      <c r="J36" s="144"/>
+      <c r="D36" s="123"/>
+      <c r="E36" s="123"/>
+      <c r="F36" s="129"/>
+      <c r="G36" s="130"/>
+      <c r="H36" s="123"/>
+      <c r="I36" s="123"/>
+      <c r="J36" s="123"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" s="161">
+      <c r="A37" s="133">
         <f>'📅 Weekly'!C15</f>
         <v>46104</v>
       </c>
-      <c r="B37" s="152">
+      <c r="B37" s="126">
         <f>ABS('📅 Weekly'!E15)</f>
         <v>0</v>
       </c>
-      <c r="C37" s="154">
+      <c r="C37" s="128">
         <f>'📅 Weekly'!F15</f>
         <v>0</v>
       </c>
-      <c r="D37" s="144"/>
-      <c r="E37" s="144"/>
-      <c r="F37" s="155"/>
-      <c r="G37" s="156"/>
-      <c r="H37" s="144"/>
-      <c r="I37" s="144"/>
-      <c r="J37" s="144"/>
+      <c r="D37" s="123"/>
+      <c r="E37" s="123"/>
+      <c r="F37" s="129"/>
+      <c r="G37" s="130"/>
+      <c r="H37" s="123"/>
+      <c r="I37" s="123"/>
+      <c r="J37" s="123"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A38" s="161">
+      <c r="A38" s="133">
         <f>'📅 Weekly'!C16</f>
         <v>46111</v>
       </c>
-      <c r="B38" s="152">
+      <c r="B38" s="126">
         <f>ABS('📅 Weekly'!E16)</f>
         <v>400.09</v>
       </c>
-      <c r="C38" s="154">
+      <c r="C38" s="128">
         <f>'📅 Weekly'!F16</f>
         <v>4</v>
       </c>
-      <c r="D38" s="144"/>
-      <c r="E38" s="144"/>
-      <c r="F38" s="155"/>
-      <c r="G38" s="156"/>
-      <c r="H38" s="144"/>
-      <c r="I38" s="144"/>
-      <c r="J38" s="144"/>
+      <c r="D38" s="123"/>
+      <c r="E38" s="123"/>
+      <c r="F38" s="129"/>
+      <c r="G38" s="130"/>
+      <c r="H38" s="123"/>
+      <c r="I38" s="123"/>
+      <c r="J38" s="123"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A39" s="161">
+      <c r="A39" s="133">
         <f>'📅 Weekly'!C17</f>
         <v>46118</v>
       </c>
-      <c r="B39" s="152">
+      <c r="B39" s="126">
         <f>ABS('📅 Weekly'!E17)</f>
         <v>95.210000000000008</v>
       </c>
-      <c r="C39" s="154">
+      <c r="C39" s="128">
         <f>'📅 Weekly'!F17</f>
         <v>3</v>
       </c>
-      <c r="D39" s="144"/>
-      <c r="E39" s="144"/>
-      <c r="F39" s="155"/>
-      <c r="G39" s="156"/>
-      <c r="H39" s="144"/>
-      <c r="I39" s="144"/>
-      <c r="J39" s="144"/>
+      <c r="D39" s="123"/>
+      <c r="E39" s="123"/>
+      <c r="F39" s="129"/>
+      <c r="G39" s="130"/>
+      <c r="H39" s="123"/>
+      <c r="I39" s="123"/>
+      <c r="J39" s="123"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A40" s="161">
+      <c r="A40" s="133">
         <f>'📅 Weekly'!C18</f>
         <v>46125</v>
       </c>
-      <c r="B40" s="152">
+      <c r="B40" s="126">
         <f>ABS('📅 Weekly'!E18)</f>
         <v>103.5</v>
       </c>
-      <c r="C40" s="154">
+      <c r="C40" s="128">
         <f>'📅 Weekly'!F18</f>
         <v>1</v>
       </c>
-      <c r="D40" s="144"/>
-      <c r="E40" s="144"/>
-      <c r="F40" s="155"/>
-      <c r="G40" s="156"/>
-      <c r="H40" s="144"/>
-      <c r="I40" s="144"/>
-      <c r="J40" s="144"/>
+      <c r="D40" s="123"/>
+      <c r="E40" s="123"/>
+      <c r="F40" s="129"/>
+      <c r="G40" s="130"/>
+      <c r="H40" s="123"/>
+      <c r="I40" s="123"/>
+      <c r="J40" s="123"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" s="161">
+      <c r="A41" s="133">
         <f>'📅 Weekly'!C19</f>
         <v>46132</v>
       </c>
-      <c r="B41" s="152">
+      <c r="B41" s="126">
         <f>ABS('📅 Weekly'!E19)</f>
         <v>1163.94</v>
       </c>
-      <c r="C41" s="154">
+      <c r="C41" s="128">
         <f>'📅 Weekly'!F19</f>
         <v>4</v>
       </c>
-      <c r="D41" s="144"/>
-      <c r="E41" s="144"/>
-      <c r="F41" s="155"/>
-      <c r="G41" s="156"/>
-      <c r="H41" s="144"/>
-      <c r="I41" s="144"/>
-      <c r="J41" s="144"/>
+      <c r="D41" s="123"/>
+      <c r="E41" s="123"/>
+      <c r="F41" s="129"/>
+      <c r="G41" s="130"/>
+      <c r="H41" s="123"/>
+      <c r="I41" s="123"/>
+      <c r="J41" s="123"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" s="161">
+      <c r="A42" s="133">
         <f>'📅 Weekly'!C20</f>
         <v>46139</v>
       </c>
-      <c r="B42" s="152">
+      <c r="B42" s="126">
         <f>ABS('📅 Weekly'!E20)</f>
         <v>677.26</v>
       </c>
-      <c r="C42" s="154">
+      <c r="C42" s="128">
         <f>'📅 Weekly'!F20</f>
         <v>5</v>
       </c>
-      <c r="D42" s="144"/>
-      <c r="E42" s="144"/>
-      <c r="F42" s="155"/>
-      <c r="G42" s="156"/>
-      <c r="H42" s="144"/>
-      <c r="I42" s="144"/>
-      <c r="J42" s="144"/>
+      <c r="D42" s="123"/>
+      <c r="E42" s="123"/>
+      <c r="F42" s="129"/>
+      <c r="G42" s="130"/>
+      <c r="H42" s="123"/>
+      <c r="I42" s="123"/>
+      <c r="J42" s="123"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" s="161">
+      <c r="A43" s="133">
         <f>'📅 Weekly'!C21</f>
         <v>46146</v>
       </c>
-      <c r="B43" s="152">
+      <c r="B43" s="126">
         <f>ABS('📅 Weekly'!E21)</f>
         <v>172.68</v>
       </c>
-      <c r="C43" s="154">
+      <c r="C43" s="128">
         <f>'📅 Weekly'!F21</f>
         <v>3</v>
       </c>
-      <c r="D43" s="144"/>
-      <c r="E43" s="144"/>
-      <c r="F43" s="155"/>
-      <c r="G43" s="156"/>
-      <c r="H43" s="144"/>
-      <c r="I43" s="144"/>
-      <c r="J43" s="144"/>
+      <c r="D43" s="123"/>
+      <c r="E43" s="123"/>
+      <c r="F43" s="129"/>
+      <c r="G43" s="130"/>
+      <c r="H43" s="123"/>
+      <c r="I43" s="123"/>
+      <c r="J43" s="123"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" s="161">
+      <c r="A44" s="133">
         <f>'📅 Weekly'!C22</f>
         <v>46153</v>
       </c>
-      <c r="B44" s="152">
+      <c r="B44" s="126">
         <f>ABS('📅 Weekly'!E22)</f>
         <v>183.67</v>
       </c>
-      <c r="C44" s="154">
+      <c r="C44" s="128">
         <f>'📅 Weekly'!F22</f>
         <v>2</v>
       </c>
-      <c r="D44" s="144"/>
-      <c r="E44" s="144"/>
-      <c r="F44" s="155"/>
-      <c r="G44" s="156"/>
-      <c r="H44" s="144"/>
-      <c r="I44" s="144"/>
-      <c r="J44" s="144"/>
+      <c r="D44" s="123"/>
+      <c r="E44" s="123"/>
+      <c r="F44" s="129"/>
+      <c r="G44" s="130"/>
+      <c r="H44" s="123"/>
+      <c r="I44" s="123"/>
+      <c r="J44" s="123"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" s="161">
+      <c r="A45" s="133">
         <f>'📅 Weekly'!C23</f>
         <v>46160</v>
       </c>
-      <c r="B45" s="152">
+      <c r="B45" s="126">
         <f>ABS('📅 Weekly'!E23)</f>
         <v>800.42</v>
       </c>
-      <c r="C45" s="154">
+      <c r="C45" s="128">
         <f>'📅 Weekly'!F23</f>
         <v>5</v>
       </c>
-      <c r="D45" s="144"/>
-      <c r="E45" s="144"/>
-      <c r="F45" s="155"/>
-      <c r="G45" s="156"/>
-      <c r="H45" s="144"/>
-      <c r="I45" s="144"/>
-      <c r="J45" s="144"/>
+      <c r="D45" s="123"/>
+      <c r="E45" s="123"/>
+      <c r="F45" s="129"/>
+      <c r="G45" s="130"/>
+      <c r="H45" s="123"/>
+      <c r="I45" s="123"/>
+      <c r="J45" s="123"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" s="161">
+      <c r="A46" s="133">
         <f>'📅 Weekly'!C24</f>
         <v>46167</v>
       </c>
-      <c r="B46" s="152">
+      <c r="B46" s="126">
         <f>ABS('📅 Weekly'!E24)</f>
         <v>317.25</v>
       </c>
-      <c r="C46" s="154">
+      <c r="C46" s="128">
         <f>'📅 Weekly'!F24</f>
         <v>3</v>
       </c>
-      <c r="D46" s="144"/>
-      <c r="E46" s="144"/>
-      <c r="F46" s="155"/>
-      <c r="G46" s="156"/>
-      <c r="H46" s="144"/>
-      <c r="I46" s="144"/>
-      <c r="J46" s="144"/>
+      <c r="D46" s="123"/>
+      <c r="E46" s="123"/>
+      <c r="F46" s="129"/>
+      <c r="G46" s="130"/>
+      <c r="H46" s="123"/>
+      <c r="I46" s="123"/>
+      <c r="J46" s="123"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" s="161">
+      <c r="A47" s="133">
         <f>'📅 Weekly'!C25</f>
         <v>46174</v>
       </c>
-      <c r="B47" s="152">
+      <c r="B47" s="126">
         <f>ABS('📅 Weekly'!E25)</f>
         <v>425.12</v>
       </c>
-      <c r="C47" s="154">
+      <c r="C47" s="128">
         <f>'📅 Weekly'!F25</f>
         <v>5</v>
       </c>
-      <c r="D47" s="144"/>
-      <c r="E47" s="144"/>
-      <c r="F47" s="155"/>
-      <c r="G47" s="156"/>
-      <c r="H47" s="144"/>
-      <c r="I47" s="144"/>
-      <c r="J47" s="144"/>
+      <c r="D47" s="123"/>
+      <c r="E47" s="123"/>
+      <c r="F47" s="129"/>
+      <c r="G47" s="130"/>
+      <c r="H47" s="123"/>
+      <c r="I47" s="123"/>
+      <c r="J47" s="123"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" s="161">
+      <c r="A48" s="133">
         <f>'📅 Weekly'!C26</f>
         <v>46181</v>
       </c>
-      <c r="B48" s="152">
+      <c r="B48" s="126">
         <f>ABS('📅 Weekly'!E26)</f>
         <v>0</v>
       </c>
-      <c r="C48" s="154">
+      <c r="C48" s="128">
         <f>'📅 Weekly'!F26</f>
         <v>0</v>
       </c>
-      <c r="D48" s="144"/>
-      <c r="E48" s="144"/>
-      <c r="F48" s="155"/>
-      <c r="G48" s="156"/>
-      <c r="H48" s="144"/>
-      <c r="I48" s="144"/>
-      <c r="J48" s="144"/>
+      <c r="D48" s="123"/>
+      <c r="E48" s="123"/>
+      <c r="F48" s="129"/>
+      <c r="G48" s="130"/>
+      <c r="H48" s="123"/>
+      <c r="I48" s="123"/>
+      <c r="J48" s="123"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" s="161">
+      <c r="A49" s="133">
         <f>'📅 Weekly'!C27</f>
         <v>46188</v>
       </c>
-      <c r="B49" s="152">
+      <c r="B49" s="126">
         <f>ABS('📅 Weekly'!E27)</f>
         <v>0</v>
       </c>
-      <c r="C49" s="154">
+      <c r="C49" s="128">
         <f>'📅 Weekly'!F27</f>
         <v>0</v>
       </c>
-      <c r="D49" s="144"/>
-      <c r="E49" s="144"/>
-      <c r="F49" s="155"/>
-      <c r="G49" s="156"/>
-      <c r="H49" s="144"/>
-      <c r="I49" s="144"/>
-      <c r="J49" s="144"/>
+      <c r="D49" s="123"/>
+      <c r="E49" s="123"/>
+      <c r="F49" s="129"/>
+      <c r="G49" s="130"/>
+      <c r="H49" s="123"/>
+      <c r="I49" s="123"/>
+      <c r="J49" s="123"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" s="161">
+      <c r="A50" s="133">
         <f>'📅 Weekly'!C28</f>
         <v>46195</v>
       </c>
-      <c r="B50" s="152">
+      <c r="B50" s="126">
         <f>ABS('📅 Weekly'!E28)</f>
         <v>0</v>
       </c>
-      <c r="C50" s="154">
+      <c r="C50" s="128">
         <f>'📅 Weekly'!F28</f>
         <v>0</v>
       </c>
-      <c r="D50" s="144"/>
-      <c r="E50" s="144"/>
-      <c r="F50" s="155"/>
-      <c r="G50" s="156"/>
-      <c r="H50" s="144"/>
-      <c r="I50" s="144"/>
-      <c r="J50" s="144"/>
+      <c r="D50" s="123"/>
+      <c r="E50" s="123"/>
+      <c r="F50" s="129"/>
+      <c r="G50" s="130"/>
+      <c r="H50" s="123"/>
+      <c r="I50" s="123"/>
+      <c r="J50" s="123"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A51" s="161">
+      <c r="A51" s="133">
         <f>'📅 Weekly'!C29</f>
         <v>46202</v>
       </c>
-      <c r="B51" s="152">
+      <c r="B51" s="126">
         <f>ABS('📅 Weekly'!E29)</f>
         <v>0</v>
       </c>
-      <c r="C51" s="154">
+      <c r="C51" s="128">
         <f>'📅 Weekly'!F29</f>
         <v>0</v>
       </c>
-      <c r="D51" s="144"/>
-      <c r="E51" s="144"/>
-      <c r="F51" s="155"/>
-      <c r="G51" s="156"/>
-      <c r="H51" s="144"/>
-      <c r="I51" s="144"/>
-      <c r="J51" s="144"/>
+      <c r="D51" s="123"/>
+      <c r="E51" s="123"/>
+      <c r="F51" s="129"/>
+      <c r="G51" s="130"/>
+      <c r="H51" s="123"/>
+      <c r="I51" s="123"/>
+      <c r="J51" s="123"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A52" s="144"/>
-      <c r="B52" s="155"/>
-      <c r="C52" s="156"/>
-      <c r="D52" s="144"/>
-      <c r="E52" s="144"/>
-      <c r="F52" s="155"/>
-      <c r="G52" s="156"/>
-      <c r="H52" s="144"/>
-      <c r="I52" s="144"/>
-      <c r="J52" s="144"/>
+      <c r="A52" s="123"/>
+      <c r="B52" s="129"/>
+      <c r="C52" s="130"/>
+      <c r="D52" s="123"/>
+      <c r="E52" s="123"/>
+      <c r="F52" s="129"/>
+      <c r="G52" s="130"/>
+      <c r="H52" s="123"/>
+      <c r="I52" s="123"/>
+      <c r="J52" s="123"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A53" s="144"/>
-      <c r="B53" s="155"/>
-      <c r="C53" s="156"/>
-      <c r="D53" s="144"/>
-      <c r="E53" s="144"/>
-      <c r="F53" s="155"/>
-      <c r="G53" s="156"/>
-      <c r="H53" s="144"/>
-      <c r="I53" s="144"/>
-      <c r="J53" s="144"/>
+      <c r="A53" s="123"/>
+      <c r="B53" s="129"/>
+      <c r="C53" s="130"/>
+      <c r="D53" s="123"/>
+      <c r="E53" s="123"/>
+      <c r="F53" s="129"/>
+      <c r="G53" s="130"/>
+      <c r="H53" s="123"/>
+      <c r="I53" s="123"/>
+      <c r="J53" s="123"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A54" s="144"/>
-      <c r="B54" s="155"/>
-      <c r="C54" s="156"/>
-      <c r="D54" s="144"/>
-      <c r="E54" s="144"/>
-      <c r="F54" s="155"/>
-      <c r="G54" s="156"/>
-      <c r="H54" s="144"/>
-      <c r="I54" s="144"/>
-      <c r="J54" s="144"/>
+      <c r="A54" s="123"/>
+      <c r="B54" s="129"/>
+      <c r="C54" s="130"/>
+      <c r="D54" s="123"/>
+      <c r="E54" s="123"/>
+      <c r="F54" s="129"/>
+      <c r="G54" s="130"/>
+      <c r="H54" s="123"/>
+      <c r="I54" s="123"/>
+      <c r="J54" s="123"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A55" s="145" t="s">
+      <c r="A55" s="134" t="s">
         <v>674</v>
       </c>
-      <c r="B55" s="157"/>
-      <c r="C55" s="158"/>
-      <c r="D55" s="144"/>
-      <c r="E55" s="144"/>
-      <c r="F55" s="155"/>
-      <c r="G55" s="156"/>
-      <c r="H55" s="144"/>
-      <c r="I55" s="144"/>
-      <c r="J55" s="144"/>
+      <c r="B55" s="135"/>
+      <c r="C55" s="137"/>
+      <c r="D55" s="123"/>
+      <c r="E55" s="123"/>
+      <c r="F55" s="129"/>
+      <c r="G55" s="130"/>
+      <c r="H55" s="123"/>
+      <c r="I55" s="123"/>
+      <c r="J55" s="123"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A56" s="150" t="s">
+      <c r="A56" s="124" t="s">
         <v>74</v>
       </c>
-      <c r="B56" s="159" t="s">
+      <c r="B56" s="131" t="s">
         <v>669</v>
       </c>
-      <c r="C56" s="160" t="s">
+      <c r="C56" s="132" t="s">
         <v>675</v>
       </c>
-      <c r="D56" s="144"/>
-      <c r="E56" s="144"/>
-      <c r="F56" s="155"/>
-      <c r="G56" s="156"/>
-      <c r="H56" s="144"/>
-      <c r="I56" s="144"/>
-      <c r="J56" s="144"/>
+      <c r="D56" s="123"/>
+      <c r="E56" s="123"/>
+      <c r="F56" s="129"/>
+      <c r="G56" s="130"/>
+      <c r="H56" s="123"/>
+      <c r="I56" s="123"/>
+      <c r="J56" s="123"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A57" s="151" t="s">
+      <c r="A57" s="125" t="s">
         <v>434</v>
       </c>
-      <c r="B57" s="152">
+      <c r="B57" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A57,'💳 MP Faturas'!D4:D149)</f>
         <v>9036.83</v>
       </c>
-      <c r="C57" s="154">
+      <c r="C57" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A57)</f>
         <v>1</v>
       </c>
-      <c r="D57" s="144"/>
-      <c r="E57" s="144"/>
-      <c r="F57" s="155"/>
-      <c r="G57" s="156"/>
-      <c r="H57" s="144"/>
-      <c r="I57" s="144"/>
-      <c r="J57" s="144"/>
+      <c r="D57" s="123"/>
+      <c r="E57" s="123"/>
+      <c r="F57" s="129"/>
+      <c r="G57" s="130"/>
+      <c r="H57" s="123"/>
+      <c r="I57" s="123"/>
+      <c r="J57" s="123"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A58" s="151" t="s">
+      <c r="A58" s="125" t="s">
         <v>400</v>
       </c>
-      <c r="B58" s="152">
+      <c r="B58" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A58,'💳 MP Faturas'!D4:D149)</f>
         <v>7395.6299999999992</v>
       </c>
-      <c r="C58" s="154">
+      <c r="C58" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A58)</f>
         <v>3</v>
       </c>
-      <c r="D58" s="144"/>
-      <c r="E58" s="144"/>
-      <c r="F58" s="155"/>
-      <c r="G58" s="156"/>
-      <c r="H58" s="144"/>
-      <c r="I58" s="144"/>
-      <c r="J58" s="144"/>
+      <c r="D58" s="123"/>
+      <c r="E58" s="123"/>
+      <c r="F58" s="129"/>
+      <c r="G58" s="130"/>
+      <c r="H58" s="123"/>
+      <c r="I58" s="123"/>
+      <c r="J58" s="123"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" s="151" t="s">
+      <c r="A59" s="125" t="s">
         <v>370</v>
       </c>
-      <c r="B59" s="152">
+      <c r="B59" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A59,'💳 MP Faturas'!D4:D149)</f>
         <v>2182.73</v>
       </c>
-      <c r="C59" s="154">
+      <c r="C59" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A59)</f>
         <v>5</v>
       </c>
-      <c r="D59" s="144"/>
-      <c r="E59" s="144"/>
-      <c r="F59" s="155"/>
-      <c r="G59" s="156"/>
-      <c r="H59" s="144"/>
-      <c r="I59" s="144"/>
-      <c r="J59" s="144"/>
+      <c r="D59" s="123"/>
+      <c r="E59" s="123"/>
+      <c r="F59" s="129"/>
+      <c r="G59" s="130"/>
+      <c r="H59" s="123"/>
+      <c r="I59" s="123"/>
+      <c r="J59" s="123"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" s="151" t="s">
+      <c r="A60" s="125" t="s">
         <v>383</v>
       </c>
-      <c r="B60" s="152">
+      <c r="B60" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A60,'💳 MP Faturas'!D4:D149)</f>
         <v>1252.3499999999999</v>
       </c>
-      <c r="C60" s="154">
+      <c r="C60" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A60)</f>
         <v>2</v>
       </c>
-      <c r="D60" s="144"/>
-      <c r="E60" s="144"/>
-      <c r="F60" s="155"/>
-      <c r="G60" s="156"/>
-      <c r="H60" s="144"/>
-      <c r="I60" s="144"/>
-      <c r="J60" s="144"/>
+      <c r="D60" s="123"/>
+      <c r="E60" s="123"/>
+      <c r="F60" s="129"/>
+      <c r="G60" s="130"/>
+      <c r="H60" s="123"/>
+      <c r="I60" s="123"/>
+      <c r="J60" s="123"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" s="151" t="s">
+      <c r="A61" s="125" t="s">
         <v>359</v>
       </c>
-      <c r="B61" s="152">
+      <c r="B61" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A61,'💳 MP Faturas'!D4:D149)</f>
         <v>1074.79</v>
       </c>
-      <c r="C61" s="154">
+      <c r="C61" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A61)</f>
         <v>10</v>
       </c>
-      <c r="D61" s="144"/>
-      <c r="E61" s="144"/>
-      <c r="F61" s="155"/>
-      <c r="G61" s="156"/>
-      <c r="H61" s="144"/>
-      <c r="I61" s="144"/>
-      <c r="J61" s="144"/>
+      <c r="D61" s="123"/>
+      <c r="E61" s="123"/>
+      <c r="F61" s="129"/>
+      <c r="G61" s="130"/>
+      <c r="H61" s="123"/>
+      <c r="I61" s="123"/>
+      <c r="J61" s="123"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A62" s="151" t="s">
+      <c r="A62" s="125" t="s">
         <v>446</v>
       </c>
-      <c r="B62" s="152">
+      <c r="B62" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A62,'💳 MP Faturas'!D4:D149)</f>
         <v>942.08</v>
       </c>
-      <c r="C62" s="154">
+      <c r="C62" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A62)</f>
         <v>4</v>
       </c>
-      <c r="D62" s="144"/>
-      <c r="E62" s="144"/>
-      <c r="F62" s="155"/>
-      <c r="G62" s="156"/>
-      <c r="H62" s="144"/>
-      <c r="I62" s="144"/>
-      <c r="J62" s="144"/>
+      <c r="D62" s="123"/>
+      <c r="E62" s="123"/>
+      <c r="F62" s="129"/>
+      <c r="G62" s="130"/>
+      <c r="H62" s="123"/>
+      <c r="I62" s="123"/>
+      <c r="J62" s="123"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" s="151" t="s">
+      <c r="A63" s="125" t="s">
         <v>501</v>
       </c>
-      <c r="B63" s="152">
+      <c r="B63" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A63,'💳 MP Faturas'!D4:D149)</f>
         <v>650.99</v>
       </c>
-      <c r="C63" s="154">
+      <c r="C63" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A63)</f>
         <v>7</v>
       </c>
-      <c r="D63" s="144"/>
-      <c r="E63" s="144"/>
-      <c r="F63" s="155"/>
-      <c r="G63" s="156"/>
-      <c r="H63" s="144"/>
-      <c r="I63" s="144"/>
-      <c r="J63" s="144"/>
+      <c r="D63" s="123"/>
+      <c r="E63" s="123"/>
+      <c r="F63" s="129"/>
+      <c r="G63" s="130"/>
+      <c r="H63" s="123"/>
+      <c r="I63" s="123"/>
+      <c r="J63" s="123"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A64" s="151" t="s">
+      <c r="A64" s="125" t="s">
         <v>507</v>
       </c>
-      <c r="B64" s="152">
+      <c r="B64" s="126">
         <f>SUMIF('💳 MP Faturas'!C4:C149,A64,'💳 MP Faturas'!D4:D149)</f>
         <v>622.66999999999996</v>
       </c>
-      <c r="C64" s="154">
+      <c r="C64" s="128">
         <f>COUNTIF('💳 MP Faturas'!C4:C149,A64)</f>
         <v>3</v>
       </c>
-      <c r="D64" s="144"/>
-      <c r="E64" s="144"/>
-      <c r="F64" s="155"/>
-      <c r="G64" s="156"/>
-      <c r="H64" s="144"/>
-      <c r="I64" s="144"/>
-      <c r="J64" s="144"/>
+      <c r="D64" s="123"/>
+      <c r="E64" s="123"/>
+      <c r="F64" s="129"/>
+      <c r="G64" s="130"/>
+      <c r="H64" s="123"/>
+      <c r="I64" s="123"/>
+      <c r="J64" s="123"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="E12:G12"/>
@@ -15988,7 +15974,28 @@
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="I8:J8"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:H9"/>
   </mergeCells>
+  <conditionalFormatting sqref="B26:B51">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{CADAF5AE-0E64-AF4F-B46D-E4FC9DA959BC}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C14:C20">
     <cfRule type="dataBar" priority="1">
       <dataBar>
@@ -16003,25 +16010,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B26:B51">
-    <cfRule type="dataBar" priority="2">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CADAF5AE-0E64-AF4F-B46D-E4FC9DA959BC}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{CADAF5AE-0E64-AF4F-B46D-E4FC9DA959BC}">
+            <x14:dataBar minLength="0" maxLength="100" direction="leftToRight" negativeBarColorSameAsPositive="1" axisPosition="none">
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>B26:B51</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{8B7E025B-3D1C-1542-BFC5-1D6A215A6C4F}">
             <x14:dataBar minLength="0" maxLength="100" direction="leftToRight" negativeBarColorSameAsPositive="1" axisPosition="none">
@@ -16030,15 +16032,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>C14:C20</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CADAF5AE-0E64-AF4F-B46D-E4FC9DA959BC}">
-            <x14:dataBar minLength="0" maxLength="100" direction="leftToRight" negativeBarColorSameAsPositive="1" axisPosition="none">
-              <x14:cfvo type="min"/>
-              <x14:cfvo type="max"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>B26:B51</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -16060,24 +16053,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
     </row>
     <row r="2" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
     </row>
     <row r="3" spans="2:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -16193,14 +16186,14 @@
       </c>
     </row>
     <row r="11" spans="2:7" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="129" t="s">
+      <c r="B11" s="149" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="124"/>
-      <c r="D11" s="124"/>
-      <c r="E11" s="124"/>
-      <c r="F11" s="124"/>
-      <c r="G11" s="124"/>
+      <c r="C11" s="144"/>
+      <c r="D11" s="144"/>
+      <c r="E11" s="144"/>
+      <c r="F11" s="144"/>
+      <c r="G11" s="144"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -16230,33 +16223,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
-      <c r="I1" s="124"/>
-      <c r="J1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
+      <c r="J1" s="144"/>
       <c r="L1" s="109" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="2" spans="2:14" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
       <c r="L2" s="110" t="s">
         <v>68</v>
       </c>
@@ -18675,37 +18668,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>173</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
-      <c r="I1" s="124"/>
-      <c r="J1" s="124"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
+      <c r="J1" s="144"/>
+      <c r="K1" s="144"/>
+      <c r="L1" s="144"/>
       <c r="N1" s="109" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="2" spans="2:16" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="124"/>
-      <c r="K2" s="124"/>
-      <c r="L2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
       <c r="N2" s="110" t="s">
         <v>68</v>
       </c>
@@ -19452,26 +19445,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>235</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
     </row>
     <row r="2" spans="2:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>236</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
     </row>
     <row r="3" spans="2:8" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -19627,24 +19620,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
     </row>
     <row r="2" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>252</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
     </row>
     <row r="3" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
@@ -20242,30 +20235,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>286</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
-      <c r="I1" s="124"/>
-      <c r="J1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
+      <c r="J1" s="144"/>
     </row>
     <row r="2" spans="2:10" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>287</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
     </row>
     <row r="3" spans="2:10" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -21205,17 +21198,17 @@
       </c>
     </row>
     <row r="37" spans="2:10" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="130" t="s">
+      <c r="B37" s="150" t="s">
         <v>317</v>
       </c>
-      <c r="C37" s="124"/>
-      <c r="D37" s="124"/>
-      <c r="E37" s="124"/>
-      <c r="F37" s="124"/>
-      <c r="G37" s="124"/>
-      <c r="H37" s="124"/>
-      <c r="I37" s="124"/>
-      <c r="J37" s="124"/>
+      <c r="C37" s="144"/>
+      <c r="D37" s="144"/>
+      <c r="E37" s="144"/>
+      <c r="F37" s="144"/>
+      <c r="G37" s="144"/>
+      <c r="H37" s="144"/>
+      <c r="I37" s="144"/>
+      <c r="J37" s="144"/>
     </row>
     <row r="38" spans="2:10" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="90">
@@ -21352,24 +21345,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>326</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
     </row>
     <row r="2" spans="2:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="143" t="s">
         <v>327</v>
       </c>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
     </row>
     <row r="3" spans="2:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -21884,11 +21877,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="146" t="s">
         <v>336</v>
       </c>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
     </row>
     <row r="3" spans="2:4" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="108" t="s">
@@ -21896,11 +21889,11 @@
       </c>
     </row>
     <row r="4" spans="2:4" ht="130" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="131" t="s">
+      <c r="B4" s="151" t="s">
         <v>338</v>
       </c>
-      <c r="C4" s="132"/>
-      <c r="D4" s="133"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="153"/>
     </row>
     <row r="6" spans="2:4" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="108" t="s">
@@ -21908,11 +21901,11 @@
       </c>
     </row>
     <row r="7" spans="2:4" ht="130" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="131" t="s">
+      <c r="B7" s="151" t="s">
         <v>340</v>
       </c>
-      <c r="C7" s="132"/>
-      <c r="D7" s="133"/>
+      <c r="C7" s="152"/>
+      <c r="D7" s="153"/>
     </row>
     <row r="9" spans="2:4" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="108" t="s">
@@ -21920,11 +21913,11 @@
       </c>
     </row>
     <row r="10" spans="2:4" ht="130" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="131" t="s">
+      <c r="B10" s="151" t="s">
         <v>342</v>
       </c>
-      <c r="C10" s="132"/>
-      <c r="D10" s="133"/>
+      <c r="C10" s="152"/>
+      <c r="D10" s="153"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>